<commit_message>
Contenidos viernes 18 de septiembre
</commit_message>
<xml_diff>
--- a/Horario.xlsx
+++ b/Horario.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daw2\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daw2\Documents\Repo DAW\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -258,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -269,6 +269,63 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -278,16 +335,10 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -296,69 +347,19 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -653,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:G18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
@@ -661,8 +662,18 @@
     <col min="8" max="8" width="5.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="36"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="36"/>
       <c r="B2" s="4"/>
       <c r="C2" s="3" t="s">
         <v>0</v>
@@ -679,251 +690,284 @@
       <c r="G2" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="36"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="36"/>
       <c r="B3" s="1">
         <v>0.625</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="21" t="s">
+      <c r="D3" s="7"/>
+      <c r="E3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="36"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="36"/>
       <c r="B4" s="2">
         <v>0.66319444444444442</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="10"/>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C4" s="6"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="36"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="36"/>
       <c r="B5" s="1">
         <v>0.66319444444444442</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="36"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="36"/>
       <c r="B6" s="2">
         <v>0.70138888888888884</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="10"/>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C6" s="6"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="36"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="36"/>
       <c r="B7" s="1">
         <v>0.70138888888888884</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="G7" s="28" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="36"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="36"/>
       <c r="B8" s="2">
         <v>0.73958333333333337</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="35"/>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C8" s="6"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="36"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="36"/>
       <c r="B9" s="1">
         <v>0.73958333333333337</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="G9" s="28" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="36"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="36"/>
       <c r="B10" s="2">
         <v>0.77777777777777779</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="35"/>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C10" s="11"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="36"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="36"/>
       <c r="B11" s="1">
         <v>0.77777777777777779</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="36"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="36"/>
       <c r="B12" s="2">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="36"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="36"/>
       <c r="B13" s="1">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="28" t="s">
+      <c r="D13" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="19" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H13" s="36"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="36"/>
       <c r="B14" s="2">
         <v>0.82638888888888884</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="12"/>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C14" s="11"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="36"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="36"/>
       <c r="B15" s="1">
         <v>0.82638888888888884</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="19" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H15" s="36"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="36"/>
       <c r="B16" s="2">
         <v>0.86458333333333337</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="12"/>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C16" s="11"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="36"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="36"/>
       <c r="B17" s="1">
         <v>0.86458333333333337</v>
       </c>
-      <c r="C17" s="27"/>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="18"/>
+      <c r="D17" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="13"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="6"/>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E17" s="30"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="36"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="36"/>
       <c r="B18" s="2">
         <v>0.90277777777777779</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="7"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="36"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="36"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="36"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="C15:C16"/>
     <mergeCell ref="G17:G18"/>
     <mergeCell ref="C11:G12"/>
     <mergeCell ref="G5:G6"/>
@@ -940,6 +984,26 @@
     <mergeCell ref="F17:F18"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>